<commit_message>
using minio for db transfer ONLY IN DEV
</commit_message>
<xml_diff>
--- a/data/Testx.xlsx
+++ b/data/Testx.xlsx
@@ -5,13 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="default" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="replacement" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="inside" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="replacement" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="inside" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -23,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -40,34 +39,13 @@
     <t xml:space="preserve">location</t>
   </si>
   <si>
-    <t xml:space="preserve">routing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">table</t>
-  </si>
-  <si>
-    <t xml:space="preserve">field</t>
-  </si>
-  <si>
-    <t xml:space="preserve">type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">timetables</t>
-  </si>
-  <si>
     <t xml:space="preserve">gong_id</t>
   </si>
   <si>
-    <t xml:space="preserve">int</t>
-  </si>
-  <si>
     <t xml:space="preserve">targets</t>
   </si>
   <si>
     <t xml:space="preserve">CC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">str</t>
   </si>
   <si>
     <t xml:space="preserve">period_type</t>
@@ -323,7 +301,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.02"/>
@@ -358,7 +336,15 @@
         <v>5</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>7012</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -373,67 +359,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -448,35 +373,35 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -490,7 +415,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -500,35 +425,35 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
corrected period cleanup + put it on every change
</commit_message>
<xml_diff>
--- a/data/Testx.xlsx
+++ b/data/Testx.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="23">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -340,7 +340,7 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -420,7 +420,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -454,6 +454,17 @@
       </c>
       <c r="C3" s="2" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cleanup of f-strings and some imports
</commit_message>
<xml_diff>
--- a/data/Testx.xlsx
+++ b/data/Testx.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="24">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -431,7 +431,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -475,6 +475,17 @@
         <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
spegoff@authentica.eu for short delay always
</commit_message>
<xml_diff>
--- a/data/Testx.xlsx
+++ b/data/Testx.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="1" state="visible" r:id="rId3"/>
@@ -33,7 +33,7 @@
     <t xml:space="preserve">timezon</t>
   </si>
   <si>
-    <t xml:space="preserve">Etc/GMT+10</t>
+    <t xml:space="preserve">Europe/Paris</t>
   </si>
   <si>
     <t xml:space="preserve">location</t>

</xml_diff>

<commit_message>
documentation-2 + cleanup pyproject.toml
</commit_message>
<xml_diff>
--- a/data/Testx.xlsx
+++ b/data/Testx.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="29">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -33,7 +33,7 @@
     <t xml:space="preserve">timezon</t>
   </si>
   <si>
-    <t xml:space="preserve">America/Chicago</t>
+    <t xml:space="preserve">Europe/Paris</t>
   </si>
   <si>
     <t xml:space="preserve">location</t>
@@ -106,6 +106,9 @@
   </si>
   <si>
     <t xml:space="preserve">Service after d0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fillin</t>
   </si>
 </sst>
 </file>
@@ -139,8 +142,9 @@
     </font>
     <font>
       <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -194,11 +198,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -222,37 +226,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -343,7 +347,7 @@
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -360,7 +364,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -372,10 +376,10 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>9</v>
       </c>
     </row>
@@ -398,41 +402,41 @@
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="14.23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="15.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="17.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="14.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="15.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="17.95"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>17</v>
       </c>
     </row>
@@ -452,45 +456,45 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.91"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>23</v>
       </c>
     </row>
@@ -506,28 +510,36 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="1" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>